<commit_message>
fix: replace stub xlsx with real seed file
</commit_message>
<xml_diff>
--- a/implementation/phase1/db_files/CRM_Datastore_Quickstart_v1.xlsx
+++ b/implementation/phase1/db_files/CRM_Datastore_Quickstart_v1.xlsx
@@ -1554,7 +1554,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M35"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1617,7 +1617,7 @@
         <v>estimator</v>
       </c>
       <c r="G2" t="str">
-        <v>in_progress</v>
+        <v>done</v>
       </c>
       <c r="H2" t="str">
         <v>2026-03-07T14:00:00Z</v>
@@ -1626,7 +1626,7 @@
         <v>2026-03-09</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>2026-03-09T07:09:31.456Z</v>
       </c>
       <c r="K2" t="str">
         <v>Set BidStatus=submitted</v>
@@ -1740,7 +1740,7 @@
         <v>estimator</v>
       </c>
       <c r="G5" t="str">
-        <v>assigned</v>
+        <v>done</v>
       </c>
       <c r="H5" t="str">
         <v>2026-03-09T03:34:02.780Z</v>
@@ -1749,7 +1749,7 @@
         <v/>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>2026-03-09T11:21:22.867Z</v>
       </c>
       <c r="K5" t="str">
         <v>Set BidStatus=submitted</v>
@@ -1843,9 +1843,1157 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ASG-0007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C8" t="str">
+        <v>WO-0001</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E8" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F8" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G8" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2026-03-09T07:09:06.455Z</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L8" t="str">
+        <v>high</v>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ASG-0008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C9" t="str">
+        <v>WO-0001</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E9" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F9" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G9" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2026-03-09T07:09:06.919Z</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L9" t="str">
+        <v>high</v>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ASG-0009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C10" t="str">
+        <v>WO-0001</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E10" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F10" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G10" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2026-03-09T07:09:07.158Z</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L10" t="str">
+        <v>high</v>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>ASG-0010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C11" t="str">
+        <v>WO-0001</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E11" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F11" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G11" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2026-03-09T07:09:15.631Z</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L11" t="str">
+        <v>high</v>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ASG-0011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>bid</v>
+      </c>
+      <c r="C12" t="str">
+        <v>BID-20260305-001</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Complete bid pricing and submit</v>
+      </c>
+      <c r="E12" t="str">
+        <v>USR-003</v>
+      </c>
+      <c r="F12" t="str">
+        <v>estimator</v>
+      </c>
+      <c r="G12" t="str">
+        <v>done</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2026-03-09T07:09:36.600Z</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v>2026-03-10T05:59:41.795Z</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Set BidStatus=submitted</v>
+      </c>
+      <c r="L12" t="str">
+        <v>medium</v>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>ASG-0012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C13" t="str">
+        <v>WO-0003</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E13" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F13" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G13" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2026-03-09T07:09:49.632Z</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L13" t="str">
+        <v>high</v>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>ASG-0013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>bid</v>
+      </c>
+      <c r="C14" t="str">
+        <v>BID-20260227-001</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Complete bid pricing and submit</v>
+      </c>
+      <c r="E14" t="str">
+        <v>USR-003</v>
+      </c>
+      <c r="F14" t="str">
+        <v>estimator</v>
+      </c>
+      <c r="G14" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2026-03-09T11:14:01.012Z</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v>Set BidStatus=submitted</v>
+      </c>
+      <c r="L14" t="str">
+        <v>medium</v>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>ASG-0014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>bid</v>
+      </c>
+      <c r="C15" t="str">
+        <v>BID-20260227-001</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Complete bid pricing and submit</v>
+      </c>
+      <c r="E15" t="str">
+        <v>USR-003</v>
+      </c>
+      <c r="F15" t="str">
+        <v>estimator</v>
+      </c>
+      <c r="G15" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2026-03-09T11:21:05.377Z</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v>Set BidStatus=submitted</v>
+      </c>
+      <c r="L15" t="str">
+        <v>medium</v>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>ASG-0015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C16" t="str">
+        <v>WO-0002</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E16" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F16" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G16" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H16" t="str">
+        <v>2026-03-09T11:21:32.321Z</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L16" t="str">
+        <v>high</v>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>ASG-0016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C17" t="str">
+        <v>WO-0002</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E17" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F17" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G17" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H17" t="str">
+        <v>2026-03-09T11:21:33.123Z</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L17" t="str">
+        <v>high</v>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>ASG-0017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C18" t="str">
+        <v>WO-0002</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E18" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F18" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G18" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H18" t="str">
+        <v>2026-03-09T11:21:33.307Z</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L18" t="str">
+        <v>high</v>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>ASG-0018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C19" t="str">
+        <v>WO-0002</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E19" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F19" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G19" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H19" t="str">
+        <v>2026-03-09T11:21:33.495Z</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L19" t="str">
+        <v>high</v>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>ASG-0019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C20" t="str">
+        <v>WO-0002</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E20" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F20" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G20" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H20" t="str">
+        <v>2026-03-09T11:21:33.714Z</v>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L20" t="str">
+        <v>high</v>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>ASG-0020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>bid</v>
+      </c>
+      <c r="C21" t="str">
+        <v>BID-20260305-001</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Complete bid pricing and submit</v>
+      </c>
+      <c r="E21" t="str">
+        <v>USR-003</v>
+      </c>
+      <c r="F21" t="str">
+        <v>estimator</v>
+      </c>
+      <c r="G21" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H21" t="str">
+        <v>2026-03-09T11:21:43.167Z</v>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v>Set BidStatus=submitted</v>
+      </c>
+      <c r="L21" t="str">
+        <v>medium</v>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>ASG-0021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>bid</v>
+      </c>
+      <c r="C22" t="str">
+        <v>BID-20260305-001</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Complete bid pricing and submit</v>
+      </c>
+      <c r="E22" t="str">
+        <v>USR-003</v>
+      </c>
+      <c r="F22" t="str">
+        <v>estimator</v>
+      </c>
+      <c r="G22" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H22" t="str">
+        <v>2026-03-09T11:21:53.174Z</v>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v>Set BidStatus=submitted</v>
+      </c>
+      <c r="L22" t="str">
+        <v>medium</v>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>ASG-0022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>bid</v>
+      </c>
+      <c r="C23" t="str">
+        <v>BID-LOCAL-0007</v>
+      </c>
+      <c r="D23" t="str">
+        <v>ROUH</v>
+      </c>
+      <c r="E23" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F23" t="str">
+        <v>estimator</v>
+      </c>
+      <c r="G23" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H23" t="str">
+        <v>2026-03-10T05:54:12.702Z</v>
+      </c>
+      <c r="I23" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v>Set BidStatus=submitted</v>
+      </c>
+      <c r="L23" t="str">
+        <v>high</v>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>ASG-0023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>bid</v>
+      </c>
+      <c r="C24" t="str">
+        <v>BID-LOCAL-0009</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Complete bid pricing and submit</v>
+      </c>
+      <c r="E24" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F24" t="str">
+        <v>estimator</v>
+      </c>
+      <c r="G24" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H24" t="str">
+        <v>2026-03-10T05:58:44.863Z</v>
+      </c>
+      <c r="I24" t="str">
+        <v>2026-03-31</v>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v>Set BidStatus=submitted</v>
+      </c>
+      <c r="L24" t="str">
+        <v>high</v>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>ASG-0024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C25" t="str">
+        <v>WO-0005</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E25" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F25" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G25" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H25" t="str">
+        <v>2026-03-10T05:59:46.917Z</v>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L25" t="str">
+        <v>high</v>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>ASG-0025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C26" t="str">
+        <v>WO-0006</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E26" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F26" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G26" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H26" t="str">
+        <v>2026-03-10T06:00:49.415Z</v>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L26" t="str">
+        <v>high</v>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>ASG-0026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C27" t="str">
+        <v>WO-0006</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E27" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F27" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G27" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H27" t="str">
+        <v>2026-03-10T06:00:55.543Z</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L27" t="str">
+        <v>high</v>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>ASG-0027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C28" t="str">
+        <v>WO-0006</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E28" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F28" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G28" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H28" t="str">
+        <v>2026-03-10T06:00:56.244Z</v>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L28" t="str">
+        <v>high</v>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>ASG-0028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C29" t="str">
+        <v>WO-0006</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Execute assigned work order</v>
+      </c>
+      <c r="E29" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F29" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G29" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H29" t="str">
+        <v>2026-03-10T06:00:56.796Z</v>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L29" t="str">
+        <v>high</v>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>ASG-0029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>bid</v>
+      </c>
+      <c r="C30" t="str">
+        <v>BID-LOCAL-0010</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Complete bid pricing and submit</v>
+      </c>
+      <c r="E30" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F30" t="str">
+        <v>estimator</v>
+      </c>
+      <c r="G30" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H30" t="str">
+        <v>2026-03-10T06:09:08.815Z</v>
+      </c>
+      <c r="I30" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v>Set BidStatus=submitted</v>
+      </c>
+      <c r="L30" t="str">
+        <v>high</v>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>ASG-0030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>general</v>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+      <c r="D31" t="str">
+        <v>New Task</v>
+      </c>
+      <c r="E31" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F31" t="str">
+        <v>general</v>
+      </c>
+      <c r="G31" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="H31" t="str">
+        <v>2026-03-12T12:17:48.291Z</v>
+      </c>
+      <c r="I31" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
+        <v/>
+      </c>
+      <c r="L31" t="str">
+        <v>medium</v>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>ASG-0031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>general</v>
+      </c>
+      <c r="C32" t="str">
+        <v/>
+      </c>
+      <c r="D32" t="str">
+        <v>fdf</v>
+      </c>
+      <c r="E32" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F32" t="str">
+        <v>general</v>
+      </c>
+      <c r="G32" t="str">
+        <v>done</v>
+      </c>
+      <c r="H32" t="str">
+        <v>2026-03-12T12:18:14.396Z</v>
+      </c>
+      <c r="I32" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="J32" t="str">
+        <v>2026-03-12T12:43:42.259Z</v>
+      </c>
+      <c r="K32" t="str">
+        <v/>
+      </c>
+      <c r="L32" t="str">
+        <v>low</v>
+      </c>
+      <c r="M32" t="str">
+        <v>fdfd</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>ASG-0032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>work_order</v>
+      </c>
+      <c r="C33" t="str">
+        <v>WO-0020</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Execute: New Work Order</v>
+      </c>
+      <c r="E33" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F33" t="str">
+        <v>installer</v>
+      </c>
+      <c r="G33" t="str">
+        <v>done</v>
+      </c>
+      <c r="H33" t="str">
+        <v>2026-03-12T12:19:17.832Z</v>
+      </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
+        <v>2026-03-12T12:21:21.020Z</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Set WorkOrderStatus=complete</v>
+      </c>
+      <c r="L33" t="str">
+        <v>high</v>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>ASG-0033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>bid_task</v>
+      </c>
+      <c r="C34" t="str">
+        <v>BT-0008</v>
+      </c>
+      <c r="D34" t="str">
+        <v>test</v>
+      </c>
+      <c r="E34" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F34" t="str">
+        <v>general</v>
+      </c>
+      <c r="G34" t="str">
+        <v>done</v>
+      </c>
+      <c r="H34" t="str">
+        <v>2026-03-12T12:40:35.482Z</v>
+      </c>
+      <c r="I34" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="J34" t="str">
+        <v>2026-03-12T12:41:00.372Z</v>
+      </c>
+      <c r="K34" t="str">
+        <v/>
+      </c>
+      <c r="L34" t="str">
+        <v>medium</v>
+      </c>
+      <c r="M34" t="str">
+        <v>dd</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>ASG-0034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>bid_task</v>
+      </c>
+      <c r="C35" t="str">
+        <v>BT-0009</v>
+      </c>
+      <c r="D35" t="str">
+        <v>ssssss</v>
+      </c>
+      <c r="E35" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F35" t="str">
+        <v>general</v>
+      </c>
+      <c r="G35" t="str">
+        <v>done</v>
+      </c>
+      <c r="H35" t="str">
+        <v>2026-03-12T12:45:36.032Z</v>
+      </c>
+      <c r="I35" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="J35" t="str">
+        <v>2026-03-12T12:46:08.131Z</v>
+      </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
+      <c r="L35" t="str">
+        <v>medium</v>
+      </c>
+      <c r="M35" t="str">
+        <v>ssssss</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2092,7 +3240,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2196,7 +3344,7 @@
         <v>USR-003</v>
       </c>
       <c r="G3" t="str">
-        <v>assigned</v>
+        <v>submitted</v>
       </c>
       <c r="H3" t="str">
         <v>2026-03-05</v>
@@ -2205,7 +3353,7 @@
         <v>2026-03-10</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>2026-03-10</v>
       </c>
       <c r="K3" t="str">
         <v/>
@@ -2237,7 +3385,7 @@
         <v>USR-003</v>
       </c>
       <c r="G4" t="str">
-        <v>draft</v>
+        <v>submitted</v>
       </c>
       <c r="H4" t="str">
         <v>2026-03-09</v>
@@ -2246,7 +3394,7 @@
         <v>2026-03-15</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>2026-03-09</v>
       </c>
       <c r="K4" t="str">
         <v/>
@@ -2255,19 +3403,347 @@
         <v/>
       </c>
       <c r="M4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>BID-LOCAL-0003</v>
+      </c>
+      <c r="B5" t="str">
+        <v>LOCAL-1773055461580</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CUST-0009</v>
+      </c>
+      <c r="D5" t="str">
+        <v>New HVAC Bid</v>
+      </c>
+      <c r="E5" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F5" t="str">
+        <v>USR-003</v>
+      </c>
+      <c r="G5" t="str">
+        <v>draft</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-03-09</v>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-03-15</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>BID-LOCAL-0004</v>
+      </c>
+      <c r="B6" t="str">
+        <v>LOCAL-1773064033292</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CUST-0010</v>
+      </c>
+      <c r="D6" t="str">
+        <v>New HVAC Bid</v>
+      </c>
+      <c r="E6" t="str">
+        <v>USR-004</v>
+      </c>
+      <c r="F6" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="G6" t="str">
+        <v>draft</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-03-09</v>
+      </c>
+      <c r="I6" t="str">
+        <v>2026-03-15</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>BID-LOCAL-0005</v>
+      </c>
+      <c r="B7" t="str">
+        <v>LOCAL-1773120477741</v>
+      </c>
+      <c r="C7" t="str">
+        <v>CUST-0002</v>
+      </c>
+      <c r="D7" t="str">
+        <v>New Bid</v>
+      </c>
+      <c r="E7" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="F7" t="str">
+        <v>USR-003</v>
+      </c>
+      <c r="G7" t="str">
+        <v>approved</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>BID-LOCAL-0006</v>
+      </c>
+      <c r="B8" t="str">
+        <v>LOCAL-1773120587693</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CUST-0001</v>
+      </c>
+      <c r="D8" t="str">
+        <v>New Bid</v>
+      </c>
+      <c r="E8" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F8" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G8" t="str">
+        <v>approved</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="I8" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>BID-LOCAL-0007</v>
+      </c>
+      <c r="B9" t="str">
+        <v>LOCAL-1773120738669</v>
+      </c>
+      <c r="C9" t="str">
+        <v>CUST-0002</v>
+      </c>
+      <c r="D9" t="str">
+        <v>seran</v>
+      </c>
+      <c r="E9" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F9" t="str">
+        <v>USR-003</v>
+      </c>
+      <c r="G9" t="str">
+        <v>approved</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="I9" t="str">
+        <v>2026-03-25</v>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>BID-LOCAL-0008</v>
+      </c>
+      <c r="B10" t="str">
+        <v>LOCAL-1773121238332</v>
+      </c>
+      <c r="C10" t="str">
+        <v>CUST-0002</v>
+      </c>
+      <c r="D10" t="str">
+        <v>seran</v>
+      </c>
+      <c r="E10" t="str">
+        <v>USR-002</v>
+      </c>
+      <c r="F10" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="G10" t="str">
+        <v>approved</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="I10" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>BID-LOCAL-0009</v>
+      </c>
+      <c r="B11" t="str">
+        <v>LOCAL-1773122289500</v>
+      </c>
+      <c r="C11" t="str">
+        <v>CUST-0001</v>
+      </c>
+      <c r="D11" t="str">
+        <v>TEST</v>
+      </c>
+      <c r="E11" t="str">
+        <v>USR-002</v>
+      </c>
+      <c r="F11" t="str">
+        <v>USR-004</v>
+      </c>
+      <c r="G11" t="str">
+        <v>approved</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="I11" t="str">
+        <v>2026-03-31</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>BID-LOCAL-0010</v>
+      </c>
+      <c r="B12" t="str">
+        <v>LOCAL-1773122621395</v>
+      </c>
+      <c r="C12" t="str">
+        <v>CUST-0001</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Test Bid</v>
+      </c>
+      <c r="E12" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="F12" t="str">
+        <v>USR-003</v>
+      </c>
+      <c r="G12" t="str">
+        <v>approved</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2317,6 +3793,9 @@
       <c r="F2" t="str">
         <v>2026-03-09</v>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
       <c r="H2" t="str">
         <v>high</v>
       </c>
@@ -2343,6 +3822,9 @@
       <c r="F3" t="str">
         <v>2026-03-10</v>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
       <c r="H3" t="str">
         <v>medium</v>
       </c>
@@ -2350,17 +3832,219 @@
         <v>Generate from template once pricing final</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>BT-0003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>BID-LOCAL-0010</v>
+      </c>
+      <c r="C4" t="str">
+        <v>GJHGHJ</v>
+      </c>
+      <c r="D4" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="E4" t="str">
+        <v>done</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="H4" t="str">
+        <v>high</v>
+      </c>
+      <c r="I4" t="str">
+        <v>IUUU</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>BT-0004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>BID-LOCAL-0010</v>
+      </c>
+      <c r="C5" t="str">
+        <v>FGJK</v>
+      </c>
+      <c r="D5" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="E5" t="str">
+        <v>todo</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>high</v>
+      </c>
+      <c r="I5" t="str">
+        <v>MNM</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>BT-0005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>BID-LOCAL-0010</v>
+      </c>
+      <c r="C6" t="str">
+        <v>YTYT</v>
+      </c>
+      <c r="D6" t="str">
+        <v>USR-002</v>
+      </c>
+      <c r="E6" t="str">
+        <v>todo</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>high</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>BT-0006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>BID-LOCAL-0008</v>
+      </c>
+      <c r="C7" t="str">
+        <v>YTYT</v>
+      </c>
+      <c r="D7" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="E7" t="str">
+        <v>todo</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>high</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>BT-0007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>BID-20260227-001</v>
+      </c>
+      <c r="C8" t="str">
+        <v>werw3</v>
+      </c>
+      <c r="D8" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="E8" t="str">
+        <v>todo</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>low</v>
+      </c>
+      <c r="I8" t="str">
+        <v>4343</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>BT-0008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>BID-20260227-001</v>
+      </c>
+      <c r="C9" t="str">
+        <v>test</v>
+      </c>
+      <c r="D9" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="E9" t="str">
+        <v>done</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="H9" t="str">
+        <v>medium</v>
+      </c>
+      <c r="I9" t="str">
+        <v>dd</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>BT-0009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>BID-20260227-001</v>
+      </c>
+      <c r="C10" t="str">
+        <v>ssssss</v>
+      </c>
+      <c r="D10" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="E10" t="str">
+        <v>done</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="H10" t="str">
+        <v>medium</v>
+      </c>
+      <c r="I10" t="str">
+        <v>ssssss</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2458,16 +4142,240 @@
         <v>Converted from bid</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>PRJ-LOCAL-0003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>LOCAL-1773122060351</v>
+      </c>
+      <c r="C4" t="str">
+        <v>BID-LOCAL-0007</v>
+      </c>
+      <c r="D4" t="str">
+        <v>CUST-0002</v>
+      </c>
+      <c r="E4" t="str">
+        <v>seran</v>
+      </c>
+      <c r="F4" t="str">
+        <v>active</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Converted from bid BID-LOCAL-0007</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PRJ-LOCAL-0004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>LOCAL-1773122418907</v>
+      </c>
+      <c r="C5" t="str">
+        <v>BID-LOCAL-0009</v>
+      </c>
+      <c r="D5" t="str">
+        <v>CUST-0001</v>
+      </c>
+      <c r="E5" t="str">
+        <v>TEST</v>
+      </c>
+      <c r="F5" t="str">
+        <v>active</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-03-31</v>
+      </c>
+      <c r="I5" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Converted from bid BID-LOCAL-0009</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>PRJ-LOCAL-0005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>LOCAL-1773122960590</v>
+      </c>
+      <c r="C6" t="str">
+        <v>BID-LOCAL-0010</v>
+      </c>
+      <c r="D6" t="str">
+        <v>CUST-0001</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Test Bid</v>
+      </c>
+      <c r="F6" t="str">
+        <v>active</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-03-20</v>
+      </c>
+      <c r="I6" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Converted from bid BID-LOCAL-0010 re</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>PRJ-LOCAL-0006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>LOCAL-1773230042654</v>
+      </c>
+      <c r="C7" t="str">
+        <v>BID-LOCAL-0008</v>
+      </c>
+      <c r="D7" t="str">
+        <v>CUST-0002</v>
+      </c>
+      <c r="E7" t="str">
+        <v>seran</v>
+      </c>
+      <c r="F7" t="str">
+        <v>active</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Converted from bid BID-LOCAL-0008</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>PRJ-LOCAL-0007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>LOCAL-1773230061470</v>
+      </c>
+      <c r="C8" t="str">
+        <v>BID-LOCAL-0010</v>
+      </c>
+      <c r="D8" t="str">
+        <v>CUST-0001</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Test Bid</v>
+      </c>
+      <c r="F8" t="str">
+        <v>active</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Converted from bid BID-LOCAL-0010</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PRJ-LOCAL-0008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>LOCAL-1773235779337</v>
+      </c>
+      <c r="C9" t="str">
+        <v>BID-LOCAL-0006</v>
+      </c>
+      <c r="D9" t="str">
+        <v>CUST-0001</v>
+      </c>
+      <c r="E9" t="str">
+        <v>New Bid</v>
+      </c>
+      <c r="F9" t="str">
+        <v>active</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Converted from bid BID-LOCAL-0006</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PRJ-LOCAL-0009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>LOCAL-1773236965237</v>
+      </c>
+      <c r="C10" t="str">
+        <v>BID-LOCAL-0005</v>
+      </c>
+      <c r="D10" t="str">
+        <v>CUST-0002</v>
+      </c>
+      <c r="E10" t="str">
+        <v>New Bid</v>
+      </c>
+      <c r="F10" t="str">
+        <v>active</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Converted from bid BID-LOCAL-0005</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2727,19 +4635,831 @@
         <v/>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>TEST1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PP-0009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>PRJ-LOCAL-0003</v>
+      </c>
+      <c r="C10" t="str">
+        <v>rough</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="str">
+        <v>in_progress</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>PP-0010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>PRJ-LOCAL-0003</v>
+      </c>
+      <c r="C11" t="str">
+        <v>trim</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>PP-0011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>PRJ-LOCAL-0003</v>
+      </c>
+      <c r="C12" t="str">
+        <v>startup</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>PP-0012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>PRJ-LOCAL-0003</v>
+      </c>
+      <c r="C13" t="str">
+        <v>warranty</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>PP-0013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>PRJ-LOCAL-0004</v>
+      </c>
+      <c r="C14" t="str">
+        <v>rough</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="str">
+        <v>in_progress</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>PP-0014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>PRJ-LOCAL-0004</v>
+      </c>
+      <c r="C15" t="str">
+        <v>trim</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>PP-0015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>PRJ-LOCAL-0004</v>
+      </c>
+      <c r="C16" t="str">
+        <v>startup</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>PP-0016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>PRJ-LOCAL-0004</v>
+      </c>
+      <c r="C17" t="str">
+        <v>warranty</v>
+      </c>
+      <c r="D17">
+        <v>4</v>
+      </c>
+      <c r="E17" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>PP-0017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>PRJ-LOCAL-0005</v>
+      </c>
+      <c r="C18" t="str">
+        <v>rough</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="str">
+        <v>in_progress</v>
+      </c>
+      <c r="F18" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>PP-0018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>PRJ-LOCAL-0005</v>
+      </c>
+      <c r="C19" t="str">
+        <v>trim</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>PP-0019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>PRJ-LOCAL-0005</v>
+      </c>
+      <c r="C20" t="str">
+        <v>startup</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+      <c r="E20" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>PP-0020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>PRJ-LOCAL-0005</v>
+      </c>
+      <c r="C21" t="str">
+        <v>warranty</v>
+      </c>
+      <c r="D21">
+        <v>4</v>
+      </c>
+      <c r="E21" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>PP-0021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>PRJ-LOCAL-0006</v>
+      </c>
+      <c r="C22" t="str">
+        <v>rough</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="str">
+        <v>in_progress</v>
+      </c>
+      <c r="F22" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>PP-0022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>PRJ-LOCAL-0006</v>
+      </c>
+      <c r="C23" t="str">
+        <v>trim</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>PP-0023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>PRJ-LOCAL-0006</v>
+      </c>
+      <c r="C24" t="str">
+        <v>startup</v>
+      </c>
+      <c r="D24">
+        <v>3</v>
+      </c>
+      <c r="E24" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>PP-0024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>PRJ-LOCAL-0006</v>
+      </c>
+      <c r="C25" t="str">
+        <v>warranty</v>
+      </c>
+      <c r="D25">
+        <v>4</v>
+      </c>
+      <c r="E25" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>PP-0025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>PRJ-LOCAL-0007</v>
+      </c>
+      <c r="C26" t="str">
+        <v>rough</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26" t="str">
+        <v>in_progress</v>
+      </c>
+      <c r="F26" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>PP-0026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>PRJ-LOCAL-0007</v>
+      </c>
+      <c r="C27" t="str">
+        <v>trim</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>PP-0027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>PRJ-LOCAL-0007</v>
+      </c>
+      <c r="C28" t="str">
+        <v>startup</v>
+      </c>
+      <c r="D28">
+        <v>3</v>
+      </c>
+      <c r="E28" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>PP-0028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>PRJ-LOCAL-0007</v>
+      </c>
+      <c r="C29" t="str">
+        <v>warranty</v>
+      </c>
+      <c r="D29">
+        <v>4</v>
+      </c>
+      <c r="E29" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>PP-0029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>PRJ-LOCAL-0008</v>
+      </c>
+      <c r="C30" t="str">
+        <v>rough</v>
+      </c>
+      <c r="D30">
+        <v>1</v>
+      </c>
+      <c r="E30" t="str">
+        <v>in_progress</v>
+      </c>
+      <c r="F30" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>PP-0030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>PRJ-LOCAL-0008</v>
+      </c>
+      <c r="C31" t="str">
+        <v>trim</v>
+      </c>
+      <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="E31" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
+      <c r="I31" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>PP-0031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>PRJ-LOCAL-0008</v>
+      </c>
+      <c r="C32" t="str">
+        <v>startup</v>
+      </c>
+      <c r="D32">
+        <v>3</v>
+      </c>
+      <c r="E32" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>PP-0032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>PRJ-LOCAL-0008</v>
+      </c>
+      <c r="C33" t="str">
+        <v>warranty</v>
+      </c>
+      <c r="D33">
+        <v>4</v>
+      </c>
+      <c r="E33" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>PP-0033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>PRJ-LOCAL-0009</v>
+      </c>
+      <c r="C34" t="str">
+        <v>rough</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34" t="str">
+        <v>in_progress</v>
+      </c>
+      <c r="F34" t="str">
+        <v>2026-03-11</v>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>PP-0034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>PRJ-LOCAL-0009</v>
+      </c>
+      <c r="C35" t="str">
+        <v>trim</v>
+      </c>
+      <c r="D35">
+        <v>2</v>
+      </c>
+      <c r="E35" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>PP-0035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>PRJ-LOCAL-0009</v>
+      </c>
+      <c r="C36" t="str">
+        <v>startup</v>
+      </c>
+      <c r="D36">
+        <v>3</v>
+      </c>
+      <c r="E36" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v>Waiting for previous phase completion</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>PP-0036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>PRJ-LOCAL-0009</v>
+      </c>
+      <c r="C37" t="str">
+        <v>warranty</v>
+      </c>
+      <c r="D37">
+        <v>4</v>
+      </c>
+      <c r="E37" t="str">
+        <v>not_started</v>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v>Waiting for previous phase completion</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2858,7 +5578,7 @@
         <v>USR-005</v>
       </c>
       <c r="H3" t="str">
-        <v>open</v>
+        <v>assigned</v>
       </c>
       <c r="I3" t="str">
         <v>2026-03-12T08:00:00Z</v>
@@ -2929,9 +5649,808 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>WO-0004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>PRJ-260302-001</v>
+      </c>
+      <c r="C5" t="str">
+        <v>PP-0001</v>
+      </c>
+      <c r="D5" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2440 Beretania HVAC - New Work Order</v>
+      </c>
+      <c r="F5" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="G5" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="H5" t="str">
+        <v>open</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N5" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>WO-0005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>PRJ-260302-001</v>
+      </c>
+      <c r="C6" t="str">
+        <v>PP-0001</v>
+      </c>
+      <c r="D6" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2440 Beretania HVAC - New Work Order</v>
+      </c>
+      <c r="F6" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="G6" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="H6" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N6" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>WO-0006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>PRJ-LOCAL-0004</v>
+      </c>
+      <c r="C7" t="str">
+        <v>PP-0001</v>
+      </c>
+      <c r="D7" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E7" t="str">
+        <v>TEST - New Work Order</v>
+      </c>
+      <c r="F7" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="G7" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="H7" t="str">
+        <v>assigned</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N7" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>WO-0007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>PRJ-LOCAL-0008</v>
+      </c>
+      <c r="C8" t="str">
+        <v>PP-0029</v>
+      </c>
+      <c r="D8" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Rough In - Default Work Order</v>
+      </c>
+      <c r="F8" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G8" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H8" t="str">
+        <v>open</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N8" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Auto-created default work order for Rough In phase</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>WO-0008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>PRJ-LOCAL-0008</v>
+      </c>
+      <c r="C9" t="str">
+        <v>PP-0030</v>
+      </c>
+      <c r="D9" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Trim - Default Work Order</v>
+      </c>
+      <c r="F9" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G9" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H9" t="str">
+        <v>open</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N9" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Auto-created default work order for Trim phase</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>WO-0009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>PRJ-LOCAL-0008</v>
+      </c>
+      <c r="C10" t="str">
+        <v>PP-0031</v>
+      </c>
+      <c r="D10" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Startup - Default Work Order</v>
+      </c>
+      <c r="F10" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G10" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H10" t="str">
+        <v>open</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N10" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Auto-created default work order for Startup phase</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>WO-0010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>PRJ-LOCAL-0008</v>
+      </c>
+      <c r="C11" t="str">
+        <v>PP-0032</v>
+      </c>
+      <c r="D11" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Warranty - Default Work Order</v>
+      </c>
+      <c r="F11" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G11" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H11" t="str">
+        <v>open</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N11" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Auto-created default work order for Warranty phase</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>WO-0011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>PRJ-LOCAL-0009</v>
+      </c>
+      <c r="C12" t="str">
+        <v>PP-0033</v>
+      </c>
+      <c r="D12" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Rough In - Default Work Order</v>
+      </c>
+      <c r="F12" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G12" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H12" t="str">
+        <v>open</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N12" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O12" t="str">
+        <v>Auto-created default work order for Rough In phase</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>WO-0012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>PRJ-LOCAL-0009</v>
+      </c>
+      <c r="C13" t="str">
+        <v>PP-0034</v>
+      </c>
+      <c r="D13" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Trim - Default Work Order</v>
+      </c>
+      <c r="F13" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G13" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H13" t="str">
+        <v>open</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N13" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Auto-created default work order for Trim phase</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>WO-0013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>PRJ-LOCAL-0009</v>
+      </c>
+      <c r="C14" t="str">
+        <v>PP-0035</v>
+      </c>
+      <c r="D14" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Startup - Default Work Order</v>
+      </c>
+      <c r="F14" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G14" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H14" t="str">
+        <v>open</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N14" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Auto-created default work order for Startup phase</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>WO-0014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>PRJ-LOCAL-0009</v>
+      </c>
+      <c r="C15" t="str">
+        <v>PP-0036</v>
+      </c>
+      <c r="D15" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Warranty - Default Work Order1</v>
+      </c>
+      <c r="F15" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G15" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H15" t="str">
+        <v>open</v>
+      </c>
+      <c r="I15" t="str">
+        <v>2026-03-13T17:51</v>
+      </c>
+      <c r="J15" t="str">
+        <v>2026-03-17T18:48</v>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N15" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Auto-created default work order for Warranty phase1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>WO-0015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>PRJ-LOCAL-0002</v>
+      </c>
+      <c r="C16" t="str">
+        <v>PP-0006</v>
+      </c>
+      <c r="D16" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E16" t="str">
+        <v>New Work Order</v>
+      </c>
+      <c r="F16" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G16" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H16" t="str">
+        <v>open</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N16" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O16" t="str">
+        <v>TEST</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>WO-0016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>PRJ-LOCAL-0005</v>
+      </c>
+      <c r="C17" t="str">
+        <v>PP-0017</v>
+      </c>
+      <c r="D17" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E17" t="str">
+        <v>New Work Order</v>
+      </c>
+      <c r="F17" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G17" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H17" t="str">
+        <v>open</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N17" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O17" t="str">
+        <v>TEST</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>WO-0017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>PRJ-LOCAL-0007</v>
+      </c>
+      <c r="C18" t="str">
+        <v>PP-0025</v>
+      </c>
+      <c r="D18" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E18" t="str">
+        <v>New Work Order</v>
+      </c>
+      <c r="F18" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G18" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H18" t="str">
+        <v>open</v>
+      </c>
+      <c r="I18" t="str">
+        <v>2026-03-10T20:10</v>
+      </c>
+      <c r="J18" t="str">
+        <v>2026-03-05T20:10</v>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N18" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O18" t="str">
+        <v>SD</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>WO-0018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>PRJ-LOCAL-0002</v>
+      </c>
+      <c r="C19" t="str">
+        <v>PP-0006</v>
+      </c>
+      <c r="D19" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E19" t="str">
+        <v>New Work Order</v>
+      </c>
+      <c r="F19" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G19" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H19" t="str">
+        <v>open</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N19" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O19" t="str">
+        <v>hhj</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>WO-0019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>PRJ-LOCAL-0006</v>
+      </c>
+      <c r="C20" t="str">
+        <v>PP-0024</v>
+      </c>
+      <c r="D20" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E20" t="str">
+        <v>New Work Order</v>
+      </c>
+      <c r="F20" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="G20" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H20" t="str">
+        <v>open</v>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N20" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>WO-0020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>PRJ-LOCAL-0009</v>
+      </c>
+      <c r="C21" t="str">
+        <v>PP-0033</v>
+      </c>
+      <c r="D21" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E21" t="str">
+        <v>New Work Order</v>
+      </c>
+      <c r="F21" t="str">
+        <v>USR-005</v>
+      </c>
+      <c r="G21" t="str">
+        <v>USR-001</v>
+      </c>
+      <c r="H21" t="str">
+        <v>complete</v>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v>pending</v>
+      </c>
+      <c r="N21" t="str">
+        <v>pending</v>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>